<commit_message>
release trust, base-clinical, immz
</commit_message>
<xml_diff>
--- a/base-clinical/StructureDefinition-sg-allergyintolerance.xlsx
+++ b/base-clinical/StructureDefinition-sg-allergyintolerance.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-04T05:53:08+00:00</t>
+    <t>2026-10-02T08:11:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>